<commit_message>
Update current master workbook to Week 22
</commit_message>
<xml_diff>
--- a/source-docs/[source-docs-current-master] WWE_2K26_Liga_System_LY2_Opening_W22_abgeschlossen.xlsx
+++ b/source-docs/[source-docs-current-master] WWE_2K26_Liga_System_LY2_Opening_W22_abgeschlossen.xlsx
@@ -21118,10 +21118,10 @@
         <v>2</v>
       </c>
       <c r="E2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -21130,7 +21130,7 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J2" t="str">
         <v>Elite Cup</v>
@@ -21150,7 +21150,7 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F3">
         <v>19</v>
@@ -21159,7 +21159,7 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I3">
         <v>57</v>
@@ -21176,16 +21176,16 @@
         <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>Cody Rhodes</v>
+        <v>Brock Lesnar</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -21194,7 +21194,7 @@
         <v>6</v>
       </c>
       <c r="I4">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J4" t="str">
         <v>Elite Cup</v>
@@ -21208,13 +21208,13 @@
         <v>4</v>
       </c>
       <c r="C5" t="str">
-        <v>Brock Lesnar</v>
+        <v>Cody Rhodes</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5">
         <v>16</v>
@@ -21223,7 +21223,7 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5">
         <v>48</v>
@@ -21246,10 +21246,10 @@
         <v>6</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -21258,7 +21258,7 @@
         <v>9</v>
       </c>
       <c r="I6">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="J6" t="str">
         <v>Sicher</v>
@@ -21278,10 +21278,10 @@
         <v>5</v>
       </c>
       <c r="E7">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -21290,7 +21290,7 @@
         <v>10</v>
       </c>
       <c r="I7">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J7" t="str">
         <v>Sicher</v>
@@ -21304,16 +21304,16 @@
         <v>7</v>
       </c>
       <c r="C8" t="str">
-        <v>Bron Breakker</v>
+        <v>CM Punk</v>
       </c>
       <c r="D8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -21322,7 +21322,7 @@
         <v>13</v>
       </c>
       <c r="I8">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J8" t="str">
         <v>Sicher</v>
@@ -21336,13 +21336,13 @@
         <v>8</v>
       </c>
       <c r="C9" t="str">
-        <v>CM Punk</v>
+        <v>Bron Breakker</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F9">
         <v>9</v>
@@ -21351,7 +21351,7 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I9">
         <v>27</v>
@@ -21374,7 +21374,7 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F10">
         <v>8</v>
@@ -21383,7 +21383,7 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I10">
         <v>24</v>
@@ -21406,7 +21406,7 @@
         <v>10</v>
       </c>
       <c r="E11">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11">
         <v>5</v>
@@ -21415,7 +21415,7 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I11">
         <v>15</v>
@@ -21432,28 +21432,28 @@
         <v>11</v>
       </c>
       <c r="C12" t="str">
-        <v>Undertaker</v>
+        <v>Triple H</v>
       </c>
       <c r="D12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E12">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F12">
         <v>3</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
         <v>19</v>
       </c>
       <c r="I12">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J12" t="str">
-        <v>Relegation nach unten</v>
+        <v>Direkter Abstieg</v>
       </c>
     </row>
     <row r="13">
@@ -21464,28 +21464,28 @@
         <v>12</v>
       </c>
       <c r="C13" t="str">
-        <v>Triple H</v>
+        <v>Undertaker</v>
       </c>
       <c r="D13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E13">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I13">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J13" t="str">
-        <v>Direkter Abstieg</v>
+        <v>Relegation nach unten</v>
       </c>
     </row>
     <row r="14">
@@ -21502,10 +21502,10 @@
         <v>1</v>
       </c>
       <c r="E14">
+        <v>23</v>
+      </c>
+      <c r="F14">
         <v>22</v>
-      </c>
-      <c r="F14">
-        <v>21</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -21514,7 +21514,7 @@
         <v>1</v>
       </c>
       <c r="I14">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J14" t="str">
         <v>Champion + direkter Aufstieg</v>
@@ -21534,7 +21534,7 @@
         <v>2</v>
       </c>
       <c r="E15">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15">
         <v>18</v>
@@ -21543,7 +21543,7 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I15">
         <v>54</v>
@@ -21560,28 +21560,28 @@
         <v>3</v>
       </c>
       <c r="C16" t="str">
-        <v>Jacob Fatu</v>
+        <v>Bronson Reed</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E16">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F16">
         <v>14</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16">
         <v>8</v>
       </c>
       <c r="I16">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J16" t="str">
-        <v>Relegation nach oben</v>
+        <v>Sicher</v>
       </c>
     </row>
     <row r="17">
@@ -21592,28 +21592,28 @@
         <v>4</v>
       </c>
       <c r="C17" t="str">
-        <v>Bronson Reed</v>
+        <v>Jacob Fatu</v>
       </c>
       <c r="D17">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E17">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F17">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I17">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J17" t="str">
-        <v>Sicher</v>
+        <v>Relegation nach oben</v>
       </c>
     </row>
     <row r="18">
@@ -21630,7 +21630,7 @@
         <v>4</v>
       </c>
       <c r="E18">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F18">
         <v>12</v>
@@ -21639,7 +21639,7 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I18">
         <v>37</v>
@@ -21662,7 +21662,7 @@
         <v>6</v>
       </c>
       <c r="E19">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F19">
         <v>11</v>
@@ -21671,7 +21671,7 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I19">
         <v>33</v>
@@ -21688,25 +21688,25 @@
         <v>7</v>
       </c>
       <c r="C20" t="str">
-        <v>Shawn Michaels</v>
+        <v>Solo Sikoa</v>
       </c>
       <c r="D20">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E20">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F20">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I20">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J20" t="str">
         <v>Sicher</v>
@@ -21720,28 +21720,28 @@
         <v>8</v>
       </c>
       <c r="C21" t="str">
-        <v>Sheamus</v>
+        <v>Shawn Michaels</v>
       </c>
       <c r="D21">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E21">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F21">
         <v>9</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21">
         <v>13</v>
       </c>
       <c r="I21">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J21" t="str">
-        <v>Relegation nach unten</v>
+        <v>Sicher</v>
       </c>
     </row>
     <row r="22">
@@ -21752,28 +21752,28 @@
         <v>9</v>
       </c>
       <c r="C22" t="str">
-        <v>Solo Sikoa</v>
+        <v>Damian Priest</v>
       </c>
       <c r="D22">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E22">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F22">
         <v>9</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22">
         <v>13</v>
       </c>
       <c r="I22">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J22" t="str">
-        <v>Sicher</v>
+        <v>Relegation nach unten</v>
       </c>
     </row>
     <row r="23">
@@ -21784,25 +21784,25 @@
         <v>10</v>
       </c>
       <c r="C23" t="str">
-        <v>Damian Priest</v>
+        <v>Sheamus</v>
       </c>
       <c r="D23">
+        <v>5</v>
+      </c>
+      <c r="E23">
+        <v>23</v>
+      </c>
+      <c r="F23">
         <v>9</v>
       </c>
-      <c r="E23">
-        <v>22</v>
-      </c>
-      <c r="F23">
-        <v>8</v>
-      </c>
       <c r="G23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I23">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J23" t="str">
         <v>Relegation nach unten</v>
@@ -21822,10 +21822,10 @@
         <v>11</v>
       </c>
       <c r="E24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -21834,7 +21834,7 @@
         <v>18</v>
       </c>
       <c r="I24">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J24" t="str">
         <v>Relegation nach unten</v>
@@ -21854,10 +21854,10 @@
         <v>12</v>
       </c>
       <c r="E25">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25">
         <v>0</v>
@@ -21866,7 +21866,7 @@
         <v>20</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J25" t="str">
         <v>Direkter Abstieg</v>
@@ -21886,10 +21886,10 @@
         <v>12</v>
       </c>
       <c r="E26">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F26">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -21898,7 +21898,7 @@
         <v>4</v>
       </c>
       <c r="I26">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J26" t="str">
         <v>Champion + direkter Aufstieg</v>
@@ -21918,7 +21918,7 @@
         <v>1</v>
       </c>
       <c r="E27">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F27">
         <v>16</v>
@@ -21927,7 +21927,7 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I27">
         <v>48</v>
@@ -21950,10 +21950,10 @@
         <v>10</v>
       </c>
       <c r="E28">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F28">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G28">
         <v>0</v>
@@ -21962,7 +21962,7 @@
         <v>7</v>
       </c>
       <c r="I28">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J28" t="str">
         <v>Relegation nach oben</v>
@@ -21982,10 +21982,10 @@
         <v>2</v>
       </c>
       <c r="E29">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F29">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G29">
         <v>0</v>
@@ -21994,7 +21994,7 @@
         <v>8</v>
       </c>
       <c r="I29">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J29" t="str">
         <v>Sicher</v>
@@ -22014,10 +22014,10 @@
         <v>11</v>
       </c>
       <c r="E30">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F30">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G30">
         <v>0</v>
@@ -22026,7 +22026,7 @@
         <v>10</v>
       </c>
       <c r="I30">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="J30" t="str">
         <v>Relegation nach unten</v>
@@ -22040,16 +22040,16 @@
         <v>6</v>
       </c>
       <c r="C31" t="str">
-        <v>Rey Mysterio</v>
+        <v>Beckielo</v>
       </c>
       <c r="D31">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F31">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G31">
         <v>0</v>
@@ -22058,10 +22058,10 @@
         <v>12</v>
       </c>
       <c r="I31">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="J31" t="str">
-        <v>Relegation nach oben</v>
+        <v>Sicher</v>
       </c>
     </row>
     <row r="32">
@@ -22072,13 +22072,13 @@
         <v>7</v>
       </c>
       <c r="C32" t="str">
-        <v>Dominik Mysterio</v>
+        <v>Rey Mysterio</v>
       </c>
       <c r="D32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F32">
         <v>10</v>
@@ -22087,13 +22087,13 @@
         <v>0</v>
       </c>
       <c r="H32">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I32">
         <v>30</v>
       </c>
       <c r="J32" t="str">
-        <v>Sicher</v>
+        <v>Relegation nach oben</v>
       </c>
     </row>
     <row r="33">
@@ -22104,13 +22104,13 @@
         <v>8</v>
       </c>
       <c r="C33" t="str">
-        <v>Beckielo</v>
+        <v>Dominik Mysterio</v>
       </c>
       <c r="D33">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E33">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F33">
         <v>10</v>
@@ -22119,7 +22119,7 @@
         <v>0</v>
       </c>
       <c r="H33">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I33">
         <v>30</v>
@@ -22142,7 +22142,7 @@
         <v>3</v>
       </c>
       <c r="E34">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F34">
         <v>9</v>
@@ -22151,7 +22151,7 @@
         <v>0</v>
       </c>
       <c r="H34">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I34">
         <v>27</v>
@@ -22168,16 +22168,16 @@
         <v>10</v>
       </c>
       <c r="C35" t="str">
-        <v>Carmelo Hayes</v>
+        <v>Ethan Page</v>
       </c>
       <c r="D35">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E35">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F35">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G35">
         <v>0</v>
@@ -22186,10 +22186,10 @@
         <v>14</v>
       </c>
       <c r="I35">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J35" t="str">
-        <v>Relegation nach unten</v>
+        <v>Sicher</v>
       </c>
     </row>
     <row r="36">
@@ -22200,13 +22200,13 @@
         <v>11</v>
       </c>
       <c r="C36" t="str">
-        <v>Ethan Page</v>
+        <v>Carmelo Hayes</v>
       </c>
       <c r="D36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E36">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F36">
         <v>8</v>
@@ -22215,13 +22215,13 @@
         <v>0</v>
       </c>
       <c r="H36">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I36">
         <v>24</v>
       </c>
       <c r="J36" t="str">
-        <v>Sicher</v>
+        <v>Relegation nach unten</v>
       </c>
     </row>
     <row r="37">
@@ -22238,7 +22238,7 @@
         <v>5</v>
       </c>
       <c r="E37">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -22247,7 +22247,7 @@
         <v>0</v>
       </c>
       <c r="H37">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I37">
         <v>6</v>
@@ -22270,10 +22270,10 @@
         <v>8</v>
       </c>
       <c r="E38">
+        <v>23</v>
+      </c>
+      <c r="F38">
         <v>22</v>
-      </c>
-      <c r="F38">
-        <v>21</v>
       </c>
       <c r="G38">
         <v>0</v>
@@ -22282,7 +22282,7 @@
         <v>1</v>
       </c>
       <c r="I38">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J38" t="str">
         <v>Champion + direkter Aufstieg</v>
@@ -22302,7 +22302,7 @@
         <v>1</v>
       </c>
       <c r="E39">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F39">
         <v>18</v>
@@ -22311,7 +22311,7 @@
         <v>0</v>
       </c>
       <c r="H39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I39">
         <v>54</v>
@@ -22334,10 +22334,10 @@
         <v>9</v>
       </c>
       <c r="E40">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F40">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G40">
         <v>0</v>
@@ -22346,7 +22346,7 @@
         <v>5</v>
       </c>
       <c r="I40">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J40" t="str">
         <v>Relegation nach oben</v>
@@ -22366,10 +22366,10 @@
         <v>2</v>
       </c>
       <c r="E41">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F41">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G41">
         <v>0</v>
@@ -22378,7 +22378,7 @@
         <v>5</v>
       </c>
       <c r="I41">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J41" t="str">
         <v>Relegation nach oben</v>
@@ -22398,10 +22398,10 @@
         <v>3</v>
       </c>
       <c r="E42">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F42">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G42">
         <v>0</v>
@@ -22410,7 +22410,7 @@
         <v>8</v>
       </c>
       <c r="I42">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J42" t="str">
         <v>Bleibt in Regional</v>
@@ -22430,7 +22430,7 @@
         <v>6</v>
       </c>
       <c r="E43">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F43">
         <v>12</v>
@@ -22439,7 +22439,7 @@
         <v>0</v>
       </c>
       <c r="H43">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I43">
         <v>36</v>
@@ -22462,10 +22462,10 @@
         <v>4</v>
       </c>
       <c r="E44">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G44">
         <v>0</v>
@@ -22474,7 +22474,7 @@
         <v>13</v>
       </c>
       <c r="I44">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J44" t="str">
         <v>Bleibt in Regional</v>
@@ -22494,10 +22494,10 @@
         <v>5</v>
       </c>
       <c r="E45">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F45">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G45">
         <v>0</v>
@@ -22506,7 +22506,7 @@
         <v>15</v>
       </c>
       <c r="I45">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J45" t="str">
         <v>Bleibt in Regional</v>
@@ -22526,7 +22526,7 @@
         <v>7</v>
       </c>
       <c r="E46">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F46">
         <v>6</v>
@@ -22535,7 +22535,7 @@
         <v>0</v>
       </c>
       <c r="H46">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I46">
         <v>18</v>
@@ -22558,7 +22558,7 @@
         <v>10</v>
       </c>
       <c r="E47">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F47">
         <v>6</v>
@@ -22567,7 +22567,7 @@
         <v>0</v>
       </c>
       <c r="H47">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I47">
         <v>18</v>
@@ -22590,7 +22590,7 @@
         <v>11</v>
       </c>
       <c r="E48">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F48">
         <v>3</v>
@@ -22599,7 +22599,7 @@
         <v>0</v>
       </c>
       <c r="H48">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I48">
         <v>9</v>
@@ -22622,7 +22622,7 @@
         <v>12</v>
       </c>
       <c r="E49">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F49">
         <v>2</v>
@@ -22631,7 +22631,7 @@
         <v>0</v>
       </c>
       <c r="H49">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I49">
         <v>6</v>
@@ -22649,7 +22649,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -22911,9 +22911,35 @@
         <v>[source-docs-current-master] WWE_2K26_Liga_System_LY2_Opening_W21_abgeschlossen.xlsx</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11">
+        <v>22</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-06-14T02:05:31.627Z</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2026-06-14T01:57:50.921Z</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+      <c r="E11">
+        <v>18</v>
+      </c>
+      <c r="F11" t="str">
+        <v>weekly-close-package-v1-week-22</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="str">
+        <v>[source-docs-current-master] WWE_2K26_Liga_System_LY2_Opening_W22_abgeschlossen.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>